<commit_message>
loại bỏ những file html của thymleaf
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/1_OtReport.xlsx
+++ b/src/main/resources/templates/1_OtReport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Java\WorkSpace\New_HR\HVV-VHR\src\main\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD4AB48A-4691-4373-B146-8DEB2A82A225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A97499C-848E-47CF-AA39-4C7EF4A3A63D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51480" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="323" xr2:uid="{15070EE6-95B8-46E9-B082-5769C0FB64A6}"/>
   </bookViews>
@@ -809,18 +809,6 @@
     <xf numFmtId="165" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="15" fillId="0" borderId="6" xfId="23" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -869,6 +857,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -878,7 +869,16 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent5" xfId="43" builtinId="46" hidden="1"/>
@@ -3624,132 +3624,132 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" customFormat="1" ht="45.75" customHeight="1" thickTop="1">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="27" t="s">
+      <c r="K1" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="L1" s="27" t="s">
+      <c r="L1" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="M1" s="11" t="s">
+      <c r="M1" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="N1" s="11" t="s">
+      <c r="N1" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="O1" s="11" t="s">
+      <c r="O1" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="P1" s="11" t="s">
+      <c r="P1" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="Q1" s="12" t="s">
+      <c r="Q1" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="R1" s="12"/>
-      <c r="S1" s="12"/>
-      <c r="T1" s="12"/>
-      <c r="U1" s="12"/>
-      <c r="V1" s="12"/>
-      <c r="W1" s="12"/>
-      <c r="X1" s="12"/>
-      <c r="Y1" s="12"/>
-      <c r="Z1" s="12"/>
-      <c r="AA1" s="12"/>
-      <c r="AB1" s="12"/>
-      <c r="AC1" s="12"/>
-      <c r="AD1" s="12"/>
-      <c r="AE1" s="12"/>
-      <c r="AF1" s="12"/>
-      <c r="AG1" s="12"/>
-      <c r="AH1" s="12"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
+      <c r="X1" s="27"/>
+      <c r="Y1" s="27"/>
+      <c r="Z1" s="27"/>
+      <c r="AA1" s="27"/>
+      <c r="AB1" s="27"/>
+      <c r="AC1" s="27"/>
+      <c r="AD1" s="27"/>
+      <c r="AE1" s="27"/>
+      <c r="AF1" s="27"/>
+      <c r="AG1" s="27"/>
+      <c r="AH1" s="27"/>
     </row>
     <row r="2" spans="1:34" customFormat="1" ht="15" customHeight="1">
-      <c r="A2" s="25"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="13" t="s">
+      <c r="A2" s="21"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
+      <c r="P2" s="23"/>
+      <c r="Q2" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="13"/>
-      <c r="S2" s="13"/>
-      <c r="T2" s="13"/>
-      <c r="U2" s="13"/>
-      <c r="V2" s="13"/>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13"/>
-      <c r="Y2" s="13"/>
-      <c r="Z2" s="14" t="s">
+      <c r="R2" s="28"/>
+      <c r="S2" s="28"/>
+      <c r="T2" s="28"/>
+      <c r="U2" s="28"/>
+      <c r="V2" s="28"/>
+      <c r="W2" s="28"/>
+      <c r="X2" s="28"/>
+      <c r="Y2" s="28"/>
+      <c r="Z2" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="AA2" s="14"/>
-      <c r="AB2" s="14"/>
-      <c r="AC2" s="14"/>
-      <c r="AD2" s="14"/>
-      <c r="AE2" s="14"/>
-      <c r="AF2" s="14"/>
-      <c r="AG2" s="14"/>
-      <c r="AH2" s="14"/>
+      <c r="AA2" s="29"/>
+      <c r="AB2" s="29"/>
+      <c r="AC2" s="29"/>
+      <c r="AD2" s="29"/>
+      <c r="AE2" s="29"/>
+      <c r="AF2" s="29"/>
+      <c r="AG2" s="29"/>
+      <c r="AH2" s="29"/>
     </row>
     <row r="3" spans="1:34" customFormat="1" ht="60">
-      <c r="A3" s="26"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
+      <c r="A3" s="22"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="26"/>
+      <c r="L3" s="26"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
       <c r="Q3" s="8" t="s">
         <v>13</v>
       </c>
@@ -4050,6 +4050,12 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="N1:N3"/>
+    <mergeCell ref="O1:O3"/>
+    <mergeCell ref="P1:P3"/>
+    <mergeCell ref="Q1:AH1"/>
+    <mergeCell ref="Q2:Y2"/>
+    <mergeCell ref="Z2:AH2"/>
     <mergeCell ref="B1:B3"/>
     <mergeCell ref="C1:C3"/>
     <mergeCell ref="D1:D3"/>
@@ -4063,12 +4069,6 @@
     <mergeCell ref="E1:E3"/>
     <mergeCell ref="K1:K3"/>
     <mergeCell ref="L1:L3"/>
-    <mergeCell ref="N1:N3"/>
-    <mergeCell ref="O1:O3"/>
-    <mergeCell ref="P1:P3"/>
-    <mergeCell ref="Q1:AH1"/>
-    <mergeCell ref="Q2:Y2"/>
-    <mergeCell ref="Z2:AH2"/>
   </mergeCells>
   <conditionalFormatting sqref="B1 B7:B15">
     <cfRule type="expression" dxfId="0" priority="5" stopIfTrue="1">

</xml_diff>